<commit_message>
n8n board refresh 2026-10-14T17:42:09Z
</commit_message>
<xml_diff>
--- a/app/reports/TSM_research.xlsx
+++ b/app/reports/TSM_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-13 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-14 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.653</v>
+        <v>0.66</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>442.085</v>
+        <v>430.385</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.093</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>5186474137.19986</v>
+        <v>5186473830.15672</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>442.085</v>
+        <v>430.385</v>
       </c>
     </row>
     <row r="38">
@@ -1508,16 +1508,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>2292862418944</v>
+        <v>2232180539392</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>32.13</v>
+        <v>31.28</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>5.06</v>
+        <v>5.07</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>3.61</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="6">
@@ -1532,16 +1532,16 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>346209419264</v>
+        <v>348187754496</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>37.154987</v>
+        <v>38.512035</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>20.883</v>
+        <v>20.993</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>6.896</v>
+        <v>6.933</v>
       </c>
     </row>
     <row r="7">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>321302528000</v>
+        <v>337962663936</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>20.70552</v>
+        <v>22.049688</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>29.84</v>
+        <v>31.516</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>5.317</v>
+        <v>5.616</v>
       </c>
     </row>
     <row r="8">
@@ -1580,16 +1580,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>65255792640</v>
+        <v>63400919040</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>88.48484999999999</v>
+        <v>88.65626</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>17.389</v>
+        <v>17.048</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>7.076</v>
+        <v>6.937</v>
       </c>
     </row>
     <row r="9">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>66171457536</v>
+        <v>64232267776</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>61.506172</v>
+        <v>61.21519</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>24.111</v>
+        <v>23.306</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>4.854</v>
+        <v>4.692</v>
       </c>
     </row>
     <row r="10">
@@ -1628,16 +1628,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>907608588288</v>
+        <v>878072299520</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>115.21739</v>
+        <v>112.69231</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>174.444</v>
+        <v>168.852</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>88.751</v>
+        <v>85.90600000000001</v>
       </c>
     </row>
     <row r="11">
@@ -1676,14 +1676,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>538363363328</v>
+        <v>521579462656</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>32.519</v>
+        <v>32.956</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>9.602</v>
+        <v>9.731</v>
       </c>
     </row>
     <row r="13">
@@ -1698,16 +1698,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>24524388352</v>
+        <v>23756341248</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>85.75889599999999</v>
+        <v>83.07313000000001</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>38.721</v>
+        <v>39.8</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>13.522</v>
+        <v>13.899</v>
       </c>
     </row>
     <row r="15">

</xml_diff>